<commit_message>
Implementação de Blocos Dinâmicos na Locação
Commit inclui alteração na classe Block, no Modelo de Planilha de Locação.xlsx que inclui as opções de usar bloco e o nome do bloco e a implementação em si do bloco no modelo de locação.
</commit_message>
<xml_diff>
--- a/Modelo Planilha de Locacao.xlsx
+++ b/Modelo Planilha de Locacao.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\msj\Documents\GitHub\pyToScriptCAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3AAF73-6A73-4C5D-BBFC-F45D1CACD630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B845770-7E02-47E6-8BA4-B1F6E7F98698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Locacao" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>nome_ponto</t>
   </si>
@@ -104,6 +104,12 @@
   </si>
   <si>
     <t>dy_anotacao</t>
+  </si>
+  <si>
+    <t>use_block</t>
+  </si>
+  <si>
+    <t>block_path</t>
   </si>
 </sst>
 </file>
@@ -227,7 +233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -268,22 +274,23 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -594,20 +601,21 @@
   <dimension ref="A1:O179"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="7.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7" style="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" style="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="2.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" style="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="3.88671875" style="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="2.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.6640625" style="17" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.44140625" style="17" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.33203125" style="17" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="2.6640625" style="14" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="7.109375" style="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" style="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" style="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2.6640625" style="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15" style="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.88671875" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="2.6640625" style="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.6640625" style="17" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.6640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.44140625" style="20" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.33203125" style="20" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="2.6640625" style="17" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -630,10 +638,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="3"/>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="19"/>
+      <c r="I1" s="15"/>
       <c r="J1" s="3"/>
       <c r="K1" s="1" t="s">
         <v>7</v>
@@ -848,8 +856,12 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="7"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="8"/>
+      <c r="H9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="8" t="b">
+        <v>0</v>
+      </c>
       <c r="J9" s="7"/>
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
@@ -865,7 +877,9 @@
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="7"/>
-      <c r="H10" s="10"/>
+      <c r="H10" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="I10" s="8"/>
       <c r="J10" s="7"/>
       <c r="K10" s="8"/>

</xml_diff>